<commit_message>
Add metrics coverage for proxy and AA maps
</commit_message>
<xml_diff>
--- a/aa/xlsx/metrics-map.xlsx
+++ b/aa/xlsx/metrics-map.xlsx
@@ -369,7 +369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Z5"/>
+  <dimension ref="B2:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.33203125" customWidth="1" min="1" max="1"/>
@@ -410,19 +410,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IF-005</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Monitoring</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>IF-005</t>
+          <t>Node.js backend, обслуживает UI, custom API, health/readiness и Prometheus metrics endpoint</t>
         </is>
       </c>
     </row>
@@ -438,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Z6"/>
+  <dimension ref="B2:Z10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.33203125" customWidth="1" min="1" max="1"/>
@@ -513,96 +501,224 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>cmdb2label backend</t>
+          <t>cmdb2label_http_requests_total</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cmdb2label_http_requests_total</t>
+          <t>counter</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>route,status</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>IF-002, IF-003, IF-005</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>counter</t>
+          <t>route, status</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Завершенные HTTP requests по классу route и status; без query, cookies, tokens, payloads</t>
+          <t>Считает завершенные HTTP requests по bounded route class и status class; alert/dashboard: Требует согласования; sensitive labels отсутствуют</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>cmdb2label backend</t>
+          <t>cmdb2label_http_request_duration_seconds</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cmdb2label_cmdbuild_requests_total</t>
+          <t>histogram</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>method,status</t>
+          <t>seconds</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>IF-002, IF-003, IF-005</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>counter</t>
+          <t>route, status, le</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Прямые CMDBuild REST calls по method и status class; без URL query или payload</t>
+          <t>Измеряет длительность HTTP requests по bounded route class и status class; alert/dashboard: Требует согласования; sensitive labels отсутствуют</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>cmdb2label backend</t>
+          <t>cmdb2label_cmdbuild_requests_total</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>counter</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>requests</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>IF-004</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>method, status</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Считает прямые consumed CMDBuild REST calls по HTTP method и status class; alert/dashboard: Требует согласования; sensitive labels отсутствуют</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>cmdb2label_cmdbuild_request_duration_seconds</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>histogram</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>IF-004</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>method, status, le</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Измеряет длительность прямых consumed CMDBuild REST calls; alert/dashboard: Требует согласования; sensitive labels отсутствуют</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
           <t>cmdb2label_cmdbuild_proxy_requests_total</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>method,status</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>counter</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Generic CMDBuild proxy calls только когда proxy явно включен; по умолчанию отключен</t>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>requests</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Отключенный generic proxy path</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>method, status</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Считает generic CMDBuild proxy calls, когда proxy явно включен; alert/dashboard: Требует согласования; inactive by default; sensitive labels отсутствуют</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cmdb2label_cmdbuild_proxy_request_duration_seconds</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>histogram</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Отключенный generic proxy path</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>method, status, le</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Измеряет длительность generic CMDBuild proxy calls, когда proxy явно включен; alert/dashboard: Требует согласования; inactive by default; sensitive labels отсутствуют</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cmdb2label_build_info</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>gauge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>constant 1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>IF-005</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>version, revision, source_state, build_mode</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Публикует safe build identity для сверки версии, revision и provenance; alert/dashboard: Требует согласования; secrets/customer payload отсутствуют</t>
         </is>
       </c>
     </row>

</xml_diff>